<commit_message>
feat: complete generic workflow engine with structured conditions, WF011/WF012, and comprehensive test suite
</commit_message>
<xml_diff>
--- a/data/AI_Agent_Workflow_Assessment (1).xlsx
+++ b/data/AI_Agent_Workflow_Assessment (1).xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -889,6 +889,90 @@
       <c r="H11" t="inlineStr">
         <is>
           <t>Performance summary with metrics, problem areas, and improvement recommendations</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WF011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Invoice Audit &amp; Overdue Processing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>User asks to audit vendor invoices and flag overdue accounts payable</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Vendor invoice ledger CSV (data/invoices.csv); overdue aging threshold (30 days)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Load vendor invoices -&gt; Filter overdue invoices &gt;30 days -&gt; Evaluate overdue exposure limit -&gt; Generate accounts payable audit report</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>If total overdue exposure &gt; $2,000, escalate to finance controller</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>read_data, filter_data, aggregate_data, llm_generate</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Detailed audit table of overdue invoices and executive aging summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WF012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Contract Compliance &amp; Clause Review</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>User asks to review vendor contract terms and verify high-risk liability clauses</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Contract agreements JSON (data/contracts.json); liability risk guidelines</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Load contract text files -&gt; Parse high-risk legal clauses -&gt; Generate compliance summary report</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>If critical risk clauses identified, flag for general counsel legal review</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>read_data, legal_clause_parser, llm_generate</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Risk classification breakdown and compliance recommendations</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1140,10 +1224,20 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Condition</t>
+          <t>Condition_Expr</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
+        <is>
+          <t>On_True</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>On_False</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>On_Error</t>
         </is>
@@ -1160,7 +1254,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Load inventory</t>
+          <t>Load inventory data</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1179,6 +1273,16 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>stop</t>
         </is>
@@ -1195,7 +1299,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Compare current stock with minimum threshold</t>
+          <t>Filter items below reorder threshold</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1214,6 +1318,16 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1230,7 +1344,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Identify low-stock products</t>
+          <t>Calculate reorder quantities</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1249,6 +1363,16 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1265,7 +1389,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Calculate reorder quantity</t>
+          <t>Aggregate restock summary</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1284,6 +1408,16 @@
         </is>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1300,7 +1434,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Generate restock list</t>
+          <t>Generate restock report</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1319,6 +1453,16 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1335,7 +1479,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Load product prices</t>
+          <t>Load internal prices</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1354,6 +1498,16 @@
         </is>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>stop</t>
         </is>
@@ -1370,7 +1524,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Match products by SKU</t>
+          <t>Load vendor prices</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1389,6 +1543,16 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>stop</t>
         </is>
@@ -1405,7 +1569,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Compare internal and vendor prices</t>
+          <t>Compare internal vs vendor prices by SKU</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1415,15 +1579,25 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>{"left_key": "sku", "right_key": "sku", "compare_fields": [{"left": "internal_price", "right": "vendor_price", "diff": "difference_absolute", "diff_pct": "difference_percentage"}]}</t>
+          <t>{"left_key": "sku", "right_key": "sku", "left_val": "internal_price", "right_val": "vendor_price"}</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>step_1.output,step_2.output</t>
+          <t>step_1.output, step_2.output</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1440,17 +1614,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Calculate percentage difference</t>
+          <t>Flag price differences exceeding threshold</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>calculator</t>
+          <t>filter_data</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>{"operations": []}</t>
+          <t>{"column": "difference_percentage", "operator": "&gt;", "value": 10.0}</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1459,6 +1633,16 @@
         </is>
       </c>
       <c r="H10" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1475,25 +1659,35 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Flag exceptions</t>
+          <t>Generate price variance report</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>filter_data</t>
+          <t>llm_generate</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>{"column": "difference_percentage", "operator": "&gt;", "value": 10.0}</t>
+          <t>{"template": "Price Variance Report"}</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>step_3.output</t>
+          <t>step_4.output</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1510,7 +1704,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Read file</t>
+          <t>Load vendor feed CSV</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1520,15 +1714,25 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>{"file_path": "data/vendor_raw_feed.csv"}</t>
+          <t>{"file_path": "data/vendor_feed.csv"}</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>file:data/vendor_raw_feed.csv</t>
+          <t>file:data/vendor_feed.csv</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>stop</t>
         </is>
@@ -1545,17 +1749,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Detect columns</t>
+          <t>Validate header format and encoding</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>calculate_metrics</t>
+          <t>filter_data</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>{"operations": []}</t>
+          <t>{"check_encoding": true}</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1564,6 +1768,16 @@
         </is>
       </c>
       <c r="H13" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1580,7 +1794,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Normalize column names</t>
+          <t>Standardize column names</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1595,10 +1809,20 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>step_2.output</t>
+          <t>step_1.output</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1615,7 +1839,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Validate required fields</t>
+          <t>Filter clean product rows</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1634,6 +1858,16 @@
         </is>
       </c>
       <c r="H15" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1673,6 +1907,16 @@
           <t>continue</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1685,7 +1929,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Produce cleaned dataset</t>
+          <t>Generate cleaned dataset report</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1704,6 +1948,16 @@
         </is>
       </c>
       <c r="H17" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1720,7 +1974,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Validate required attributes</t>
+          <t>Validate required product attributes</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1739,6 +1993,16 @@
         </is>
       </c>
       <c r="H18" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1755,7 +2019,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Create product description</t>
+          <t>Generate product description</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1775,7 +2039,17 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>retry:2</t>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>continue</t>
         </is>
       </c>
     </row>
@@ -1813,6 +2087,16 @@
           <t>continue</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1825,7 +2109,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Generate SEO title</t>
+          <t>Generate SEO title (max 60 chars)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1844,6 +2128,16 @@
         </is>
       </c>
       <c r="H21" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1860,7 +2154,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Generate meta description</t>
+          <t>Generate meta description (max 160 chars)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1879,6 +2173,16 @@
         </is>
       </c>
       <c r="H22" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1895,7 +2199,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Validate identifier</t>
+          <t>Validate order identifier present</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1913,7 +2217,22 @@
           <t>params</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>identifier_present</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>ask_user</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -1930,7 +2249,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Search order data</t>
+          <t>Search order database</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1949,6 +2268,16 @@
         </is>
       </c>
       <c r="H24" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
         <is>
           <t>stop</t>
         </is>
@@ -1965,7 +2294,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Retrieve order status</t>
+          <t>Retrieve order by identifier</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1983,7 +2312,22 @@
           <t>step_2.output</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>found</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>ask_user</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2000,7 +2344,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Retrieve shipment information</t>
+          <t>Extract shipment details</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2019,6 +2363,16 @@
         </is>
       </c>
       <c r="H26" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2035,7 +2389,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Summarize current status</t>
+          <t>Summarize order status</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2054,6 +2408,16 @@
         </is>
       </c>
       <c r="H27" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2070,7 +2434,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Load products</t>
+          <t>Load product catalog</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2089,6 +2453,16 @@
         </is>
       </c>
       <c r="H28" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
         <is>
           <t>stop</t>
         </is>
@@ -2105,7 +2479,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Normalize names/SKUs</t>
+          <t>Normalize names and SKUs</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2124,6 +2498,16 @@
         </is>
       </c>
       <c r="H29" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2140,7 +2524,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Compare identifiers</t>
+          <t>Compare SKU identifiers for exact duplicates</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2159,6 +2543,16 @@
         </is>
       </c>
       <c r="H30" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2175,7 +2569,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Compare product attributes</t>
+          <t>Calculate title similarity scores</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2185,15 +2579,25 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>{"key_field": "product_name", "threshold": 0.8}</t>
+          <t>{"key_field": "product_name", "threshold": 0.85}</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>step_3.output</t>
+          <t>step_2.output</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2210,17 +2614,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Group likely duplicates</t>
+          <t>Flag potential duplicate pairs</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>aggregate_data</t>
+          <t>filter_data</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>{"aggregations": {"count": "count"}}</t>
+          <t>{"column": "similarity_score", "operator": "&gt;=", "value": 0.85}</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2229,6 +2633,16 @@
         </is>
       </c>
       <c r="H32" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2245,7 +2659,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Assign confidence</t>
+          <t>Assign duplication confidence scores</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2264,6 +2678,16 @@
         </is>
       </c>
       <c r="H33" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2280,7 +2704,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Validate inputs</t>
+          <t>Validate campaign inputs</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2298,7 +2722,22 @@
           <t>params</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>campaign_goal_present and dates_present</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>ask_user</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2338,6 +2777,16 @@
           <t>continue</t>
         </is>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2350,7 +2799,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Summarize products</t>
+          <t>Load product catalog for context</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2369,6 +2818,16 @@
         </is>
       </c>
       <c r="H36" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2385,7 +2844,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Create messaging</t>
+          <t>Create messaging pillars</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2404,6 +2863,16 @@
         </is>
       </c>
       <c r="H37" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2443,6 +2912,16 @@
           <t>continue</t>
         </is>
       </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2455,7 +2934,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Create campaign checklist</t>
+          <t>Create campaign launch checklist</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2474,6 +2953,16 @@
         </is>
       </c>
       <c r="H39" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2490,7 +2979,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Read keywords</t>
+          <t>Read keyword list</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2509,6 +2998,16 @@
         </is>
       </c>
       <c r="H40" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
         <is>
           <t>stop</t>
         </is>
@@ -2525,7 +3024,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Remove duplicates</t>
+          <t>Remove duplicate keywords</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2544,6 +3043,16 @@
         </is>
       </c>
       <c r="H41" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2583,6 +3092,16 @@
           <t>continue</t>
         </is>
       </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2595,7 +3114,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Map keywords to categories</t>
+          <t>Map keywords to page categories</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2614,6 +3133,16 @@
         </is>
       </c>
       <c r="H43" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2630,7 +3159,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Identify high-priority keywords</t>
+          <t>Identify high-priority keywords (volume &gt;= 1000)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2649,6 +3178,16 @@
         </is>
       </c>
       <c r="H44" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2665,7 +3204,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Export results</t>
+          <t>Export keyword classification report</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2684,6 +3223,16 @@
         </is>
       </c>
       <c r="H45" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2700,7 +3249,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Understand task requirements</t>
+          <t>Parse task skill requirements</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2718,7 +3267,22 @@
           <t>params</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>skills_provided</t>
+        </is>
+      </c>
       <c r="H46" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>ask_user</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2735,7 +3299,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Compare employee skills</t>
+          <t>Load employee roster</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2754,6 +3318,16 @@
         </is>
       </c>
       <c r="H47" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
         <is>
           <t>stop</t>
         </is>
@@ -2770,7 +3344,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Check current workload</t>
+          <t>Filter by matching skills and capacity</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2788,7 +3362,22 @@
           <t>step_2.output</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>qualified_count &gt; 0 and available_count &gt; 0</t>
+        </is>
+      </c>
       <c r="H48" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>escalate</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2805,7 +3394,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Rank candidates</t>
+          <t>Rank candidates by available capacity</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2824,6 +3413,16 @@
         </is>
       </c>
       <c r="H49" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2840,7 +3439,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Select employee</t>
+          <t>Select top candidate</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2859,6 +3458,16 @@
         </is>
       </c>
       <c r="H50" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2875,7 +3484,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Generate assignment summary</t>
+          <t>Generate task assignment summary</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2894,6 +3503,16 @@
         </is>
       </c>
       <c r="H51" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2910,7 +3529,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Load execution logs</t>
+          <t>Load workflow execution logs</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2929,6 +3548,16 @@
         </is>
       </c>
       <c r="H52" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
         <is>
           <t>stop</t>
         </is>
@@ -2945,7 +3574,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Calculate success/failure rate</t>
+          <t>Calculate success/failure rates per workflow</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2964,6 +3593,16 @@
         </is>
       </c>
       <c r="H53" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -2980,7 +3619,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Calculate average execution time</t>
+          <t>Calculate average execution times</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2999,6 +3638,16 @@
         </is>
       </c>
       <c r="H54" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -3015,7 +3664,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Identify frequent errors</t>
+          <t>Identify failed executions</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3034,6 +3683,16 @@
         </is>
       </c>
       <c r="H55" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -3050,7 +3709,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Identify slow steps</t>
+          <t>Identify slow steps (&gt;5s)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3069,6 +3728,16 @@
         </is>
       </c>
       <c r="H56" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
         <is>
           <t>continue</t>
         </is>
@@ -3085,7 +3754,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Generate recommendations</t>
+          <t>Generate performance recommendations</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3104,6 +3773,336 @@
         </is>
       </c>
       <c r="H57" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>WF011</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Load vendor invoice ledger</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>read_data</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>{"file_path": "data/invoices.csv"}</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>file:data/invoices.csv</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>WF011</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Filter overdue invoices (&gt;30 days)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>filter_data</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>{"column": "days_overdue", "operator": "&gt;", "value": 30}</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>step_1.output</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>WF011</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>3</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Evaluate overdue exposure limit</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>aggregate_data</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>{"aggregations": {"total_overdue": "sum:amount", "overdue_count": "count"}}</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>step_2.output</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>total_overdue &lt;= 2000</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>escalate</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>WF011</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Generate accounts payable audit report</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>llm_generate</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>{"template": "Invoice Audit"}</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>step_3.output</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>WF012</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Load contract text files</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>read_data</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>{"file_path": "data/contracts.json"}</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>file:data/contracts.json</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>WF012</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Parse high-risk legal clauses</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>legal_clause_parser</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>{"target_clause": "liability", "flag_risk": "CRITICAL"}</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>step_1.output</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>WF012</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>3</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Generate compliance summary report</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>llm_generate</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>{"template": "Compliance Review"}</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>step_2.output</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
         <is>
           <t>continue</t>
         </is>

</xml_diff>